<commit_message>
Pushing Mainboard Split Up
Mainboard will be obsoleted soon

Battery Board and Flight Controller created

Battery Board - Good amount of routing done, additional area will be used for SuperCaps
</commit_message>
<xml_diff>
--- a/Backplane/Backplane Pin Count.xlsx
+++ b/Backplane/Backplane Pin Count.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shane\Documents\GitHub\inspireFly-pocketqubeBoards\Backplane\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5034A00-6058-4285-8E75-6391AF5559E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3229D8E-FF28-4764-8878-54E512A3BC3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4110" yWindow="-21600" windowWidth="26010" windowHeight="20985" xr2:uid="{6870E42B-97D7-476E-8CD7-6F0EB1D79D9E}"/>
+    <workbookView xWindow="-4125" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{6870E42B-97D7-476E-8CD7-6F0EB1D79D9E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="52">
   <si>
     <t>PIN NAME</t>
   </si>
@@ -189,6 +189,9 @@
   </si>
   <si>
     <t>RFM_RESET</t>
+  </si>
+  <si>
+    <t>BATMANG_INT_DIN</t>
   </si>
 </sst>
 </file>
@@ -654,11 +657,11 @@
       <c r="G2" s="3"/>
       <c r="I2" s="3">
         <f>COUNTIF(C2:C42,"x")</f>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J2" s="3">
         <f>COUNTIF(D2:D36,"x")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K2" s="3">
         <f>COUNTIF(E2:E36,"x")</f>
@@ -727,11 +730,11 @@
       <c r="G4" s="3"/>
       <c r="I4" s="3">
         <f>I2 + 7</f>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J4" s="3">
         <f>J2+16</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K4" s="3">
         <f>K2+9</f>
@@ -796,10 +799,10 @@
       <c r="F6" s="4"/>
       <c r="G6" s="3"/>
       <c r="I6" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J6" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" s="3">
         <v>0</v>
@@ -1287,10 +1290,18 @@
       <c r="G33" s="3"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A34" s="2"/>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
+      <c r="A34" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>

</xml_diff>

<commit_message>
Board sizes for FC and routing. slight Backplane changes
</commit_message>
<xml_diff>
--- a/Backplane/Backplane Pin Count.xlsx
+++ b/Backplane/Backplane Pin Count.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shane\Documents\GitHub\inspireFly-pocketqubeBoards\Backplane\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3229D8E-FF28-4764-8878-54E512A3BC3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE70547-6801-4669-8F28-5E5B2247A328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4125" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{6870E42B-97D7-476E-8CD7-6F0EB1D79D9E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{6870E42B-97D7-476E-8CD7-6F0EB1D79D9E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="53">
   <si>
     <t>PIN NAME</t>
   </si>
@@ -192,6 +192,9 @@
   </si>
   <si>
     <t>BATMANG_INT_DIN</t>
+  </si>
+  <si>
+    <t>SUPER_CAP_CHARGE</t>
   </si>
 </sst>
 </file>
@@ -657,11 +660,11 @@
       <c r="G2" s="3"/>
       <c r="I2" s="3">
         <f>COUNTIF(C2:C42,"x")</f>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J2" s="3">
         <f>COUNTIF(D2:D36,"x")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K2" s="3">
         <f>COUNTIF(E2:E36,"x")</f>
@@ -730,10 +733,10 @@
       <c r="G4" s="3"/>
       <c r="I4" s="3">
         <f>I2 + 7</f>
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J4" s="3">
-        <f>J2+16</f>
+        <f>J2+15</f>
         <v>26</v>
       </c>
       <c r="K4" s="3">
@@ -799,7 +802,7 @@
       <c r="F6" s="4"/>
       <c r="G6" s="3"/>
       <c r="I6" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J6" s="3">
         <v>0</v>
@@ -1307,10 +1310,18 @@
       <c r="G34" s="3"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A35" s="2"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
+      <c r="A35" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>

</xml_diff>